<commit_message>
Add Module 4: CTEs for aggregation and joins
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -711,10 +711,10 @@
     <t xml:space="preserve">Cohorts</t>
   </si>
   <si>
-    <t xml:space="preserve">Group customers by signup year and show how many placed their first order within 30 days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">first_orders CTE with MIN(order_date)</t>
+    <t xml:space="preserve">Group customers by signup year: customers, how many ordered, average days from signup to first order, and how many ordered within 365 days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">first_orders CTE with MIN(order_date); check the distribution before choosing a threshold</t>
   </si>
   <si>
     <t xml:space="preserve">04-aggregation-patterns/04-04.sql</t>

</xml_diff>

<commit_message>
Add Module 6: data cleaning and deduplication
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -810,10 +810,10 @@
     <t xml:space="preserve">Profiling</t>
   </si>
   <si>
-    <t xml:space="preserve">Flag rows with blank names, missing emails or malformed emails.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASE + regex operator ~</t>
+    <t xml:space="preserve">Flag rows with blank names, missing emails, malformed emails or formatting problems, as one readable issues column.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASE + regex operator ~; concat_ws skips NULLs</t>
   </si>
   <si>
     <t xml:space="preserve">06-data-cleaning/06-02.sql</t>
@@ -825,10 +825,10 @@
     <t xml:space="preserve">Data-quality summary</t>
   </si>
   <si>
-    <t xml:space="preserve">One-row summary: total rows, distinct emails, duplicate rows, rows with missing name.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Several small CTEs cross-joined</t>
+    <t xml:space="preserve">One-row summary: total rows, distinct emails, duplicate rows, rows with missing name, rows with missing or malformed email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean once in a CTE, then aggregate with FILTER</t>
   </si>
   <si>
     <t xml:space="preserve">06-data-cleaning/06-03.sql</t>
@@ -13206,7 +13206,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="n">
         <v>6</v>
       </c>
@@ -13232,7 +13232,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="n">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Add Module 7: materialization and the optimizer
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -840,10 +840,10 @@
     <t xml:space="preserve">MATERIALIZED</t>
   </si>
   <si>
-    <t xml:space="preserve">Compare EXPLAIN ANALYZE for a CTE referenced twice with MATERIALIZED vs NOT MATERIALIZED.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Look for CTE Scan vs inlined scans</t>
+    <t xml:space="preserve">Compare EXPLAIN ANALYZE for a CTE referenced twice with MATERIALIZED vs NOT MATERIALIZED; count the scans of order_items in each plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Look for CTE Scan vs inlined scans; count scan nodes</t>
   </si>
   <si>
     <t xml:space="preserve">07-materialization/07-01.sql</t>
@@ -870,10 +870,10 @@
     <t xml:space="preserve">When to force</t>
   </si>
   <si>
-    <t xml:space="preserve">Document two cases where MATERIALIZED is the right choice (expensive reused computation, volatile functions).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Try random() inside a CTE referenced twice</t>
+    <t xml:space="preserve">Show three situations: a volatile random() CTE, an expensive aggregate used twice, and the opposite case where NOT MATERIALIZED wins (two selective lookups).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The hint does not override volatile functions; compare rows read</t>
   </si>
   <si>
     <t xml:space="preserve">07-materialization/07-03.sql</t>
@@ -13275,7 +13275,7 @@
         <v>266</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>97</v>
+        <v>185</v>
       </c>
       <c r="G29" s="15" t="s">
         <v>267</v>
@@ -13327,7 +13327,7 @@
         <v>276</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>30</v>
+        <v>185</v>
       </c>
       <c r="G31" s="15" t="s">
         <v>277</v>

</xml_diff>

<commit_message>
Add Module 8: UNION vs UNION ALL
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -903,10 +903,10 @@
     <t xml:space="preserve">Calendar</t>
   </si>
   <si>
-    <t xml:space="preserve">Build every date in 2026 recursively and left join orders to find days with zero orders.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gap-filling pattern</t>
+    <t xml:space="preserve">Build a recursive calendar from the first to the last order date, left join the orders to find days with zero orders, summarise by month and reconcile the totals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gap-filling pattern; take the bounds from the data, not a fixed year</t>
   </si>
   <si>
     <t xml:space="preserve">08-recursive-basics/08-02.sql</t>
@@ -933,10 +933,10 @@
     <t xml:space="preserve">Termination</t>
   </si>
   <si>
-    <t xml:space="preserve">Remove the stop condition on a small recursion in a safe sandbox (use statement_timeout) and explain what happens.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SET statement_timeout = '2s'</t>
+    <t xml:space="preserve">Run a recursion with no stop condition under statement_timeout and show it is cancelled; then compare how UNION and UNION ALL end a cycle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SET statement_timeout; catch query_canceled explicitly</t>
   </si>
   <si>
     <t xml:space="preserve">08-recursive-basics/08-04.sql</t>
@@ -13362,7 +13362,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Add Module 9: hierarchies, org charts and category trees
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -948,10 +948,10 @@
     <t xml:space="preserve">Org chart</t>
   </si>
   <si>
-    <t xml:space="preserve">List all employees under the CEO with their depth level.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">depth + 1 in the recursive member</t>
+    <t xml:space="preserve">List all employees under the CEO with their depth level, then reconcile: employees reached vs employees in total.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">depth + 1 in the recursive member; compare reached with COUNT(*)</t>
   </si>
   <si>
     <t xml:space="preserve">09-hierarchies/09-01.sql</t>
@@ -978,10 +978,10 @@
     <t xml:space="preserve">Subtree</t>
   </si>
   <si>
-    <t xml:space="preserve">All direct and indirect reports of a chosen manager, plus headcount per manager.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Start the anchor at the chosen emp_id</t>
+    <t xml:space="preserve">All direct and indirect reports of a chosen manager, plus direct and total headcount for every manager.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor at the chosen emp_id; use a closure (anchor on every reporting line) for headcounts</t>
   </si>
   <si>
     <t xml:space="preserve">09-hierarchies/09-03.sql</t>
@@ -13440,7 +13440,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="n">
         <v>9</v>
       </c>
@@ -13492,7 +13492,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="n">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Harden CI: repo check, clearer failures, LF line endings, pinned runner
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -1041,10 +1041,10 @@
     <t xml:space="preserve">Path enumeration</t>
   </si>
   <si>
-    <t xml:space="preserve">Find all routes from Nairobi to Kigali with total distance, first without cycle protection.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observe the infinite loop; use statement_timeout</t>
+    <t xml:space="preserve">Enumerate walks from Nairobi without cycle protection: observe the runaway under statement_timeout, then see why a depth limit alone reports 202 routes to Kigali when only 2 exist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor on the start node; catch query_canceled; a depth guard counts loops</t>
   </si>
   <si>
     <t xml:space="preserve">10-graphs-and-cycles/10-01.sql</t>
@@ -1086,10 +1086,10 @@
     <t xml:space="preserve">SEARCH clause</t>
   </si>
   <si>
-    <t xml:space="preserve">Order results with SEARCH BREADTH FIRST and DEPTH FIRST and explain the difference.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEARCH ... SET ordercol</t>
+    <t xml:space="preserve">Order results with SEARCH BREADTH FIRST and DEPTH FIRST, explain the difference, and show why the BY columns must make every row unique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEARCH ... SET ordercol; BREADTH FIRST BY a unique path of ids</t>
   </si>
   <si>
     <t xml:space="preserve">10-graphs-and-cycles/10-04.sql</t>
@@ -13596,7 +13596,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Add Module 11: bill of materials and roll-ups
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -1131,10 +1131,10 @@
     <t xml:space="preserve">Cost roll-up</t>
   </si>
   <si>
-    <t xml:space="preserve">Compute the total unit cost of one Bicycle.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Join exploded quantities to unit_cost</t>
+    <t xml:space="preserve">Compute the total unit cost of one Bicycle and the rolled-up cost of every assembly, then cross-check two independent ways.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Join exploded quantities to unit_cost; a closure rolls up every assembly at once</t>
   </si>
   <si>
     <t xml:space="preserve">11-bill-of-materials/11-02.sql</t>
@@ -1146,10 +1146,10 @@
     <t xml:space="preserve">Where-used</t>
   </si>
   <si>
-    <t xml:space="preserve">Find every assembly that directly or indirectly uses Bolt (recurse upwards).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swap the join direction</t>
+    <t xml:space="preserve">Find every assembly that directly or indirectly uses Bolt (recurse upwards), with the bolts each consumes, and cross-check against the downward explosion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swap the join direction; multiply quantities on the way up</t>
   </si>
   <si>
     <t xml:space="preserve">11-bill-of-materials/11-03.sql</t>
@@ -13752,7 +13752,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="n">
         <v>11</v>
       </c>
@@ -13778,7 +13778,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="n">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Add Module 13: Performance,Best Practices & Anti-Patterns, with data-safety checks
</commit_message>
<xml_diff>
--- a/docs/CTE_Explained_Beginner_to_Advanced.xlsx
+++ b/docs/CTE_Explained_Beginner_to_Advanced.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="856">
   <si>
     <t xml:space="preserve">CTE Explained: From Beginner to Advanced</t>
   </si>
@@ -1248,10 +1248,13 @@
     <t xml:space="preserve">Indexing</t>
   </si>
   <si>
-    <t xml:space="preserve">Add an index on employees(manager_id), then compare EXPLAIN ANALYZE of the org-chart recursion before and after (use a larger generated dataset).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Index the join column of the recursive step</t>
+    <t xml:space="preserve">Generate a 111,111-person org chart and traverse the whole organisation and one small team, with and without an index on manager_id; report whole-table scans vs index lookups from the plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generated big_org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Index the join column; selective traversals gain most; run ANALYZE</t>
   </si>
   <si>
     <t xml:space="preserve">13-best-practices/13-02.sql</t>
@@ -1278,10 +1281,10 @@
     <t xml:space="preserve">Alternatives</t>
   </si>
   <si>
-    <t xml:space="preserve">Write a comparison of recursive CTEs vs ltree vs closure table vs materialized path for hierarchies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read vs write cost, constraints, tooling</t>
+    <t xml:space="preserve">Build the category tree as an adjacency list, materialized path, closure table and ltree; compare reads, the rows changed by moving a subtree, and storage; then write a recommendation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read vs write cost, constraints, tooling; handle the moved node when using subpath</t>
   </si>
   <si>
     <t xml:space="preserve">13-best-practices/13-04.sql</t>
@@ -3710,16 +3713,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,7 +3730,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>3</v>
@@ -3741,7 +3744,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>3</v>
@@ -3755,7 +3758,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>3</v>
@@ -3769,7 +3772,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>4</v>
@@ -3783,7 +3786,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>4</v>
@@ -3797,7 +3800,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>6</v>
@@ -3811,7 +3814,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>6</v>
@@ -3825,7 +3828,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>6</v>
@@ -3839,7 +3842,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>7</v>
@@ -3853,7 +3856,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>7</v>
@@ -3867,7 +3870,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>7</v>
@@ -3881,7 +3884,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>7</v>
@@ -3895,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>7</v>
@@ -3909,7 +3912,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>7</v>
@@ -3923,7 +3926,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>10</v>
@@ -3937,7 +3940,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>10</v>
@@ -3951,7 +3954,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>11</v>
@@ -3965,7 +3968,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>11</v>
@@ -3979,7 +3982,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>12</v>
@@ -3993,7 +3996,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>12</v>
@@ -4033,19 +4036,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4059,7 +4062,7 @@
         <v>45658</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>5</v>
@@ -4076,7 +4079,7 @@
         <v>45663</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0</v>
@@ -4093,7 +4096,7 @@
         <v>45669</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>0</v>
@@ -4110,7 +4113,7 @@
         <v>45678</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>15</v>
@@ -4127,7 +4130,7 @@
         <v>45685</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
@@ -4144,7 +4147,7 @@
         <v>45697</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>5</v>
@@ -4161,7 +4164,7 @@
         <v>45698</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>5</v>
@@ -4178,7 +4181,7 @@
         <v>45700</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>15</v>
@@ -4195,7 +4198,7 @@
         <v>45703</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>5</v>
@@ -4212,7 +4215,7 @@
         <v>45710</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>15</v>
@@ -4229,7 +4232,7 @@
         <v>45711</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>10</v>
@@ -4246,7 +4249,7 @@
         <v>45713</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>0</v>
@@ -4263,7 +4266,7 @@
         <v>45716</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>15</v>
@@ -4280,7 +4283,7 @@
         <v>45717</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>0</v>
@@ -4297,7 +4300,7 @@
         <v>45718</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>0</v>
@@ -4314,7 +4317,7 @@
         <v>45723</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>10</v>
@@ -4331,7 +4334,7 @@
         <v>45728</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E18" s="4" t="n">
         <v>5</v>
@@ -4348,7 +4351,7 @@
         <v>45728</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>10</v>
@@ -4365,7 +4368,7 @@
         <v>45728</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>0</v>
@@ -4382,7 +4385,7 @@
         <v>45729</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>10</v>
@@ -4399,7 +4402,7 @@
         <v>45730</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>10</v>
@@ -4416,7 +4419,7 @@
         <v>45732</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>0</v>
@@ -4433,7 +4436,7 @@
         <v>45732</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>5</v>
@@ -4450,7 +4453,7 @@
         <v>45737</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>5</v>
@@ -4467,7 +4470,7 @@
         <v>45738</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>15</v>
@@ -4484,7 +4487,7 @@
         <v>45751</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>0</v>
@@ -4501,7 +4504,7 @@
         <v>45758</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>0</v>
@@ -4518,7 +4521,7 @@
         <v>45763</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>15</v>
@@ -4535,7 +4538,7 @@
         <v>45764</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E30" s="4" t="n">
         <v>5</v>
@@ -4552,7 +4555,7 @@
         <v>45766</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>10</v>
@@ -4569,7 +4572,7 @@
         <v>45767</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E32" s="4" t="n">
         <v>5</v>
@@ -4586,7 +4589,7 @@
         <v>45785</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>10</v>
@@ -4603,7 +4606,7 @@
         <v>45808</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E34" s="4" t="n">
         <v>5</v>
@@ -4620,7 +4623,7 @@
         <v>45809</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>0</v>
@@ -4637,7 +4640,7 @@
         <v>45810</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>10</v>
@@ -4654,7 +4657,7 @@
         <v>45816</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>5</v>
@@ -4671,7 +4674,7 @@
         <v>45821</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E38" s="4" t="n">
         <v>15</v>
@@ -4688,7 +4691,7 @@
         <v>45823</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>0</v>
@@ -4705,7 +4708,7 @@
         <v>45825</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E40" s="4" t="n">
         <v>0</v>
@@ -4722,7 +4725,7 @@
         <v>45827</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>15</v>
@@ -4739,7 +4742,7 @@
         <v>45829</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E42" s="4" t="n">
         <v>0</v>
@@ -4756,7 +4759,7 @@
         <v>45836</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>10</v>
@@ -4773,7 +4776,7 @@
         <v>45839</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E44" s="4" t="n">
         <v>0</v>
@@ -4790,7 +4793,7 @@
         <v>45852</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E45" s="4" t="n">
         <v>5</v>
@@ -4807,7 +4810,7 @@
         <v>45854</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E46" s="4" t="n">
         <v>15</v>
@@ -4824,7 +4827,7 @@
         <v>45855</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E47" s="4" t="n">
         <v>10</v>
@@ -4841,7 +4844,7 @@
         <v>45861</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E48" s="4" t="n">
         <v>5</v>
@@ -4858,7 +4861,7 @@
         <v>45863</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
@@ -4875,7 +4878,7 @@
         <v>45867</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E50" s="4" t="n">
         <v>10</v>
@@ -4892,7 +4895,7 @@
         <v>45873</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E51" s="4" t="n">
         <v>5</v>
@@ -4909,7 +4912,7 @@
         <v>45876</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E52" s="4" t="n">
         <v>5</v>
@@ -4926,7 +4929,7 @@
         <v>45877</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E53" s="4" t="n">
         <v>15</v>
@@ -4943,7 +4946,7 @@
         <v>45881</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E54" s="4" t="n">
         <v>10</v>
@@ -4960,7 +4963,7 @@
         <v>45882</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E55" s="4" t="n">
         <v>15</v>
@@ -4977,7 +4980,7 @@
         <v>45888</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E56" s="4" t="n">
         <v>0</v>
@@ -4994,7 +4997,7 @@
         <v>45893</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E57" s="4" t="n">
         <v>0</v>
@@ -5011,7 +5014,7 @@
         <v>45894</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E58" s="4" t="n">
         <v>5</v>
@@ -5028,7 +5031,7 @@
         <v>45898</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E59" s="4" t="n">
         <v>5</v>
@@ -5045,7 +5048,7 @@
         <v>45900</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E60" s="4" t="n">
         <v>15</v>
@@ -5062,7 +5065,7 @@
         <v>45902</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E61" s="4" t="n">
         <v>0</v>
@@ -5079,7 +5082,7 @@
         <v>45910</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E62" s="4" t="n">
         <v>0</v>
@@ -5096,7 +5099,7 @@
         <v>45911</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E63" s="4" t="n">
         <v>10</v>
@@ -5113,7 +5116,7 @@
         <v>45911</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E64" s="4" t="n">
         <v>0</v>
@@ -5130,7 +5133,7 @@
         <v>45912</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E65" s="4" t="n">
         <v>0</v>
@@ -5147,7 +5150,7 @@
         <v>45913</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E66" s="4" t="n">
         <v>0</v>
@@ -5164,7 +5167,7 @@
         <v>45924</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E67" s="4" t="n">
         <v>5</v>
@@ -5181,7 +5184,7 @@
         <v>45925</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E68" s="4" t="n">
         <v>10</v>
@@ -5198,7 +5201,7 @@
         <v>45926</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E69" s="4" t="n">
         <v>15</v>
@@ -5215,7 +5218,7 @@
         <v>45927</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E70" s="4" t="n">
         <v>15</v>
@@ -5232,7 +5235,7 @@
         <v>45927</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>5</v>
@@ -5249,7 +5252,7 @@
         <v>45928</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E72" s="4" t="n">
         <v>10</v>
@@ -5266,7 +5269,7 @@
         <v>45931</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E73" s="4" t="n">
         <v>10</v>
@@ -5283,7 +5286,7 @@
         <v>45937</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E74" s="4" t="n">
         <v>0</v>
@@ -5300,7 +5303,7 @@
         <v>45943</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>0</v>
@@ -5317,7 +5320,7 @@
         <v>45943</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E76" s="4" t="n">
         <v>15</v>
@@ -5334,7 +5337,7 @@
         <v>45948</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E77" s="4" t="n">
         <v>10</v>
@@ -5351,7 +5354,7 @@
         <v>45966</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E78" s="4" t="n">
         <v>0</v>
@@ -5368,7 +5371,7 @@
         <v>45972</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E79" s="4" t="n">
         <v>5</v>
@@ -5385,7 +5388,7 @@
         <v>45977</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E80" s="4" t="n">
         <v>15</v>
@@ -5402,7 +5405,7 @@
         <v>45985</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E81" s="4" t="n">
         <v>0</v>
@@ -5419,7 +5422,7 @@
         <v>45987</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E82" s="4" t="n">
         <v>15</v>
@@ -5436,7 +5439,7 @@
         <v>45997</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E83" s="4" t="n">
         <v>0</v>
@@ -5453,7 +5456,7 @@
         <v>45998</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E84" s="4" t="n">
         <v>15</v>
@@ -5470,7 +5473,7 @@
         <v>46003</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E85" s="4" t="n">
         <v>15</v>
@@ -5487,7 +5490,7 @@
         <v>46005</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E86" s="4" t="n">
         <v>0</v>
@@ -5504,7 +5507,7 @@
         <v>46018</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E87" s="4" t="n">
         <v>15</v>
@@ -5521,7 +5524,7 @@
         <v>46040</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E88" s="4" t="n">
         <v>15</v>
@@ -5538,7 +5541,7 @@
         <v>46051</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E89" s="4" t="n">
         <v>5</v>
@@ -5555,7 +5558,7 @@
         <v>46052</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E90" s="4" t="n">
         <v>15</v>
@@ -5572,7 +5575,7 @@
         <v>46057</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E91" s="4" t="n">
         <v>15</v>
@@ -5589,7 +5592,7 @@
         <v>46063</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E92" s="4" t="n">
         <v>10</v>
@@ -5606,7 +5609,7 @@
         <v>46066</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E93" s="4" t="n">
         <v>5</v>
@@ -5623,7 +5626,7 @@
         <v>46068</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E94" s="4" t="n">
         <v>5</v>
@@ -5640,7 +5643,7 @@
         <v>46072</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E95" s="4" t="n">
         <v>15</v>
@@ -5657,7 +5660,7 @@
         <v>46076</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E96" s="4" t="n">
         <v>10</v>
@@ -5674,7 +5677,7 @@
         <v>46083</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E97" s="4" t="n">
         <v>15</v>
@@ -5691,7 +5694,7 @@
         <v>46087</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E98" s="4" t="n">
         <v>10</v>
@@ -5708,7 +5711,7 @@
         <v>46087</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E99" s="4" t="n">
         <v>5</v>
@@ -5725,7 +5728,7 @@
         <v>46089</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E100" s="4" t="n">
         <v>0</v>
@@ -5742,7 +5745,7 @@
         <v>46095</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E101" s="4" t="n">
         <v>0</v>
@@ -5759,7 +5762,7 @@
         <v>46096</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E102" s="4" t="n">
         <v>15</v>
@@ -5776,7 +5779,7 @@
         <v>46099</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E103" s="4" t="n">
         <v>15</v>
@@ -5793,7 +5796,7 @@
         <v>46102</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E104" s="4" t="n">
         <v>10</v>
@@ -5810,7 +5813,7 @@
         <v>46103</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E105" s="4" t="n">
         <v>0</v>
@@ -5827,7 +5830,7 @@
         <v>46104</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E106" s="4" t="n">
         <v>5</v>
@@ -5844,7 +5847,7 @@
         <v>46106</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E107" s="4" t="n">
         <v>10</v>
@@ -5861,7 +5864,7 @@
         <v>46111</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E108" s="4" t="n">
         <v>15</v>
@@ -5878,7 +5881,7 @@
         <v>46114</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="E109" s="4" t="n">
         <v>15</v>
@@ -5895,7 +5898,7 @@
         <v>46129</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E110" s="4" t="n">
         <v>5</v>
@@ -5912,7 +5915,7 @@
         <v>46133</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E111" s="4" t="n">
         <v>10</v>
@@ -5929,7 +5932,7 @@
         <v>46142</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E112" s="4" t="n">
         <v>5</v>
@@ -5946,7 +5949,7 @@
         <v>46156</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E113" s="4" t="n">
         <v>10</v>
@@ -5963,7 +5966,7 @@
         <v>46158</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E114" s="4" t="n">
         <v>10</v>
@@ -5980,7 +5983,7 @@
         <v>46177</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E115" s="4" t="n">
         <v>5</v>
@@ -5997,7 +6000,7 @@
         <v>46181</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E116" s="4" t="n">
         <v>5</v>
@@ -6014,7 +6017,7 @@
         <v>46181</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E117" s="4" t="n">
         <v>5</v>
@@ -6031,7 +6034,7 @@
         <v>46191</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E118" s="4" t="n">
         <v>5</v>
@@ -6048,7 +6051,7 @@
         <v>46199</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E119" s="4" t="n">
         <v>10</v>
@@ -6065,7 +6068,7 @@
         <v>46201</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="E120" s="4" t="n">
         <v>0</v>
@@ -6082,7 +6085,7 @@
         <v>46203</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E121" s="4" t="n">
         <v>5</v>
@@ -6118,19 +6121,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11024,16 +11027,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11041,10 +11044,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>160</v>
@@ -11055,10 +11058,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>150</v>
@@ -11069,10 +11072,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>400</v>
@@ -11083,10 +11086,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>480</v>
@@ -11097,10 +11100,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>530</v>
@@ -11111,10 +11114,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>270</v>
@@ -11125,10 +11128,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>800</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>799</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>798</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>630</v>
@@ -11139,10 +11142,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>180</v>
@@ -11153,10 +11156,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>380</v>
@@ -11167,10 +11170,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>510</v>
@@ -11181,10 +11184,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>650</v>
@@ -11195,10 +11198,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>880</v>
@@ -11233,13 +11236,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11247,7 +11250,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C2" s="4"/>
     </row>
@@ -11256,7 +11259,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C3" s="4"/>
     </row>
@@ -11265,7 +11268,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C4" s="4"/>
     </row>
@@ -11274,7 +11277,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="C5" s="4"/>
     </row>
@@ -11283,7 +11286,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="C6" s="4"/>
     </row>
@@ -11292,7 +11295,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>18</v>
@@ -11303,7 +11306,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>12</v>
@@ -11314,7 +11317,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>0.25</v>
@@ -11325,7 +11328,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>15</v>
@@ -11336,7 +11339,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>9</v>
@@ -11347,7 +11350,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="C12" s="4"/>
     </row>
@@ -11356,7 +11359,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>6</v>
@@ -11367,7 +11370,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>14</v>
@@ -11378,7 +11381,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>11</v>
@@ -11389,7 +11392,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>2</v>
@@ -11400,7 +11403,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>7</v>
@@ -11411,7 +11414,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>0.1</v>
@@ -11422,7 +11425,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>60</v>
@@ -11433,7 +11436,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>10</v>
@@ -11444,7 +11447,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>8</v>
@@ -11479,13 +11482,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11738,16 +11741,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11755,10 +11758,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="D2" s="28" t="n">
         <v>46027.3333333333</v>
@@ -11769,10 +11772,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="D3" s="28" t="n">
         <v>46063.3958333333</v>
@@ -11783,10 +11786,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="D4" s="28" t="n">
         <v>46028.3333333333</v>
@@ -11797,10 +11800,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="D5" s="28" t="n">
         <v>46082.46875</v>
@@ -11811,10 +11814,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D6" s="28" t="n">
         <v>46029.3333333333</v>
@@ -11825,10 +11828,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D7" s="28" t="n">
         <v>46030.3333333333</v>
@@ -11839,10 +11842,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="D8" s="28" t="n">
         <v>46061.3333333333</v>
@@ -11853,10 +11856,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="D9" s="28" t="n">
         <v>46031.3333333333</v>
@@ -11868,7 +11871,7 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="D10" s="28" t="n">
         <v>46032.3333333333</v>
@@ -11879,10 +11882,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D11" s="28" t="n">
         <v>46033.3333333333</v>
@@ -11893,7 +11896,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="28" t="n">
@@ -11905,10 +11908,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="D13" s="28" t="n">
         <v>46035.3333333333</v>
@@ -11919,10 +11922,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="D14" s="28" t="n">
         <v>46095.6979166667</v>
@@ -11933,10 +11936,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="D15" s="28" t="n">
         <v>46037.3333333333</v>
@@ -11947,10 +11950,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="D16" s="28" t="n">
         <v>46038.3333333333</v>
@@ -11961,10 +11964,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="D17" s="28" t="n">
         <v>46039.3333333333</v>
@@ -11975,10 +11978,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="D18" s="28" t="n">
         <v>46070.3333333333</v>
@@ -11989,10 +11992,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="D19" s="28" t="n">
         <v>46040.3333333333</v>
@@ -12003,10 +12006,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="D20" s="28" t="n">
         <v>46041.3333333333</v>
@@ -12017,10 +12020,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="D21" s="28" t="n">
         <v>46100.3333333333</v>
@@ -13937,7 +13940,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="n">
         <v>13</v>
       </c>
@@ -13954,13 +13957,13 @@
         <v>402</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>22</v>
+        <v>403</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13968,51 +13971,51 @@
         <v>13</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C56" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F56" s="15" t="s">
         <v>143</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="n">
         <v>13</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C57" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F57" s="15" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14020,25 +14023,25 @@
         <v>14</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C58" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F58" s="15" t="s">
         <v>74</v>
       </c>
       <c r="G58" s="15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14046,25 +14049,25 @@
         <v>14</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C59" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F59" s="15" t="s">
         <v>69</v>
       </c>
       <c r="G59" s="15" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14072,25 +14075,25 @@
         <v>14</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C60" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F60" s="15" t="s">
         <v>386</v>
       </c>
       <c r="G60" s="15" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14098,25 +14101,25 @@
         <v>14</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C61" s="19" t="s">
         <v>45</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F61" s="15" t="s">
         <v>34</v>
       </c>
       <c r="G61" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H61" s="15" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -14149,56 +14152,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14206,223 +14209,223 @@
         <v>167</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -14451,29 +14454,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14481,16 +14484,16 @@
         <v>20</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14498,16 +14501,16 @@
         <v>20</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14515,14 +14518,14 @@
         <v>20</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14530,16 +14533,16 @@
         <v>22</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14547,16 +14550,16 @@
         <v>22</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14564,16 +14567,16 @@
         <v>22</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14581,14 +14584,14 @@
         <v>22</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="15" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14596,16 +14599,16 @@
         <v>22</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14613,16 +14616,16 @@
         <v>22</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14630,14 +14633,14 @@
         <v>22</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="15" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14645,14 +14648,14 @@
         <v>22</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="15" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14660,16 +14663,16 @@
         <v>24</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14677,16 +14680,16 @@
         <v>24</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14694,14 +14697,14 @@
         <v>24</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D18" s="15"/>
       <c r="E18" s="15" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14709,14 +14712,14 @@
         <v>24</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="15" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14724,14 +14727,14 @@
         <v>24</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D20" s="15"/>
       <c r="E20" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14739,16 +14742,16 @@
         <v>26</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14756,16 +14759,16 @@
         <v>26</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14773,16 +14776,16 @@
         <v>26</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14790,16 +14793,16 @@
         <v>28</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14807,16 +14810,16 @@
         <v>28</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14824,16 +14827,16 @@
         <v>28</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14841,14 +14844,14 @@
         <v>28</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="15" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14856,16 +14859,16 @@
         <v>30</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14873,16 +14876,16 @@
         <v>30</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14890,14 +14893,14 @@
         <v>30</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D30" s="15"/>
       <c r="E30" s="15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14905,14 +14908,14 @@
         <v>30</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="15" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14920,14 +14923,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D32" s="15"/>
       <c r="E32" s="15" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14935,16 +14938,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14952,16 +14955,16 @@
         <v>32</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14969,16 +14972,16 @@
         <v>32</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14986,14 +14989,14 @@
         <v>32</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D36" s="15"/>
       <c r="E36" s="15" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15001,14 +15004,14 @@
         <v>32</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D37" s="15"/>
       <c r="E37" s="15" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15016,16 +15019,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15033,16 +15036,16 @@
         <v>34</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15050,16 +15053,16 @@
         <v>34</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15067,14 +15070,14 @@
         <v>34</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D41" s="15"/>
       <c r="E41" s="15" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15082,16 +15085,16 @@
         <v>36</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15099,16 +15102,16 @@
         <v>36</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15116,14 +15119,14 @@
         <v>36</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D44" s="15"/>
       <c r="E44" s="15" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15131,16 +15134,16 @@
         <v>38</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15148,16 +15151,16 @@
         <v>38</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15165,16 +15168,16 @@
         <v>38</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15182,16 +15185,16 @@
         <v>40</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15199,14 +15202,14 @@
         <v>40</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D49" s="15"/>
       <c r="E49" s="15" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15214,14 +15217,14 @@
         <v>40</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D50" s="15"/>
       <c r="E50" s="15" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15229,66 +15232,66 @@
         <v>40</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="15" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="15" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C52" s="15"/>
       <c r="D52" s="15"/>
       <c r="E52" s="15" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C53" s="15"/>
       <c r="D53" s="15"/>
       <c r="E53" s="15" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C54" s="15"/>
       <c r="D54" s="15"/>
       <c r="E54" s="15" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="15" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C55" s="15"/>
       <c r="D55" s="15"/>
       <c r="E55" s="15" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
   </sheetData>
@@ -15319,13 +15322,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15333,10 +15336,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15344,10 +15347,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>628</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15355,10 +15358,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15366,10 +15369,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15377,10 +15380,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15388,10 +15391,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15399,10 +15402,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
     </row>
   </sheetData>
@@ -15439,28 +15442,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="G1" s="25" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="H1" s="25" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15468,13 +15471,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>1</v>
@@ -15492,13 +15495,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>2</v>
@@ -15518,13 +15521,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>3</v>
@@ -15544,13 +15547,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>4</v>
@@ -15570,13 +15573,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>5</v>
@@ -15596,13 +15599,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>6</v>
@@ -15622,13 +15625,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>2</v>
@@ -15648,13 +15651,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>657</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>656</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>2</v>
@@ -15674,13 +15677,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>3</v>
@@ -15700,13 +15703,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>661</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>662</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>660</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
@@ -15726,13 +15729,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>4</v>
@@ -15752,13 +15755,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>5</v>
@@ -15778,13 +15781,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>6</v>
@@ -15804,13 +15807,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
@@ -15830,13 +15833,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>677</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>675</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>676</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>674</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>2</v>
@@ -15856,13 +15859,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>2</v>
@@ -15882,13 +15885,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E18" s="4" t="n">
         <v>2</v>
@@ -15908,13 +15911,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>2</v>
@@ -15934,13 +15937,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>3</v>
@@ -15960,13 +15963,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>690</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>691</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>689</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>690</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>688</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>3</v>
@@ -15986,13 +15989,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>3</v>
@@ -16012,13 +16015,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>694</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>693</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>3</v>
@@ -16038,13 +16041,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>4</v>
@@ -16064,13 +16067,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>4</v>
@@ -16090,13 +16093,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>5</v>
@@ -16116,13 +16119,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>6</v>
@@ -16142,13 +16145,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>6</v>
@@ -16168,13 +16171,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>6</v>
@@ -16194,13 +16197,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E30" s="4" t="n">
         <v>6</v>
@@ -16220,13 +16223,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>6</v>
@@ -16272,19 +16275,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16292,13 +16295,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E2" s="27" t="n">
         <v>45581</v>
@@ -16309,13 +16312,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E3" s="27" t="n">
         <v>45177</v>
@@ -16326,13 +16329,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>726</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>725</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>726</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>724</v>
       </c>
       <c r="E4" s="27" t="n">
         <v>45619</v>
@@ -16343,13 +16346,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E5" s="27" t="n">
         <v>45531</v>
@@ -16360,13 +16363,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E6" s="27" t="n">
         <v>45022</v>
@@ -16377,13 +16380,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E7" s="27" t="n">
         <v>45501</v>
@@ -16394,13 +16397,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E8" s="27" t="n">
         <v>45152</v>
@@ -16411,13 +16414,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E9" s="27" t="n">
         <v>44933</v>
@@ -16428,13 +16431,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E10" s="27" t="n">
         <v>45641</v>
@@ -16445,13 +16448,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E11" s="27" t="n">
         <v>45086</v>
@@ -16462,13 +16465,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E12" s="27" t="n">
         <v>45031</v>
@@ -16479,13 +16482,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E13" s="27" t="n">
         <v>45294</v>
@@ -16496,13 +16499,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E14" s="27" t="n">
         <v>44971</v>
@@ -16513,13 +16516,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E15" s="27" t="n">
         <v>45314</v>
@@ -16530,13 +16533,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E16" s="27" t="n">
         <v>45570</v>
@@ -16547,13 +16550,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E17" s="27" t="n">
         <v>45518</v>
@@ -16564,13 +16567,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E18" s="27" t="n">
         <v>44973</v>
@@ -16581,13 +16584,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E19" s="27" t="n">
         <v>45008</v>
@@ -16598,13 +16601,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E20" s="27" t="n">
         <v>45316</v>
@@ -16615,13 +16618,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E21" s="27" t="n">
         <v>45093</v>
@@ -16632,13 +16635,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E22" s="27" t="n">
         <v>45613</v>
@@ -16649,13 +16652,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E23" s="27" t="n">
         <v>45550</v>
@@ -16666,13 +16669,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E24" s="27" t="n">
         <v>45094</v>
@@ -16683,13 +16686,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E25" s="27" t="n">
         <v>45582</v>
@@ -16700,13 +16703,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E26" s="27" t="n">
         <v>45628</v>
@@ -16717,13 +16720,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E27" s="27" t="n">
         <v>45161</v>
@@ -16734,13 +16737,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E28" s="27" t="n">
         <v>46133</v>
@@ -16751,13 +16754,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E29" s="27" t="n">
         <v>46154</v>
@@ -16768,13 +16771,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E30" s="27" t="n">
         <v>46109</v>
@@ -16785,13 +16788,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E31" s="27" t="n">
         <v>46164</v>
@@ -16826,13 +16829,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16840,7 +16843,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C2" s="4"/>
     </row>
@@ -16849,7 +16852,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>1</v>
@@ -16860,7 +16863,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>2</v>
@@ -16871,7 +16874,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>2</v>
@@ -16882,7 +16885,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>1</v>
@@ -16893,7 +16896,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>5</v>
@@ -16904,7 +16907,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>1</v>
@@ -16915,7 +16918,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="C9" s="4"/>
     </row>
@@ -16924,7 +16927,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>8</v>
@@ -16935,7 +16938,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>9</v>
@@ -16946,7 +16949,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>9</v>
@@ -16957,7 +16960,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>8</v>

</xml_diff>